<commit_message>
📊 Actualización manual del dashboard
</commit_message>
<xml_diff>
--- a/Comentarios Campaña.xlsx
+++ b/Comentarios Campaña.xlsx
@@ -19,11 +19,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -54,10 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -504,6 +501,11 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>extraction_status</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>created_time_raw</t>
         </is>
       </c>
@@ -545,7 +547,7 @@
       <c r="H2" s="1" t="n">
         <v>46211.58980324074</v>
       </c>
-      <c r="I2" s="2" t="n">
+      <c r="I2" s="1" t="n">
         <v>46211</v>
       </c>
       <c r="J2" t="inlineStr">
@@ -568,7 +570,8 @@
           <t>https://instagram.com/mat18545</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>{'postUrl': 'https://www.instagram.com/p/DZ5yxYgAy5c/', 'commentUrl': 'https://www.instagram.com/p/DZ5yxYgAy5c/c/18197756167366742', 'id': '18197756167366742', 'text': 'Vuelvan a los animales marinos por favor', 'ownerUsername': 'mat18545', 'ownerProfilePicUrl': 'https://scontent-bru2-1.cdninstagram.com/v/t51.2885-19/469370398_1109721463381756_4068535561865210393_n.jpg?stp=dst-jpg_e0_s150x150_tt6&amp;_nc_cat=103&amp;ig_cache_key=GB4G_hv83p8pSfEDABkqBZmJV3Y4bkULAAAB1501500j-ccb7-5&amp;ccb=7-5&amp;_nc_sid=669407&amp;</t>
         </is>
@@ -611,7 +614,7 @@
       <c r="H3" s="1" t="n">
         <v>46210.59957175926</v>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="I3" s="1" t="n">
         <v>46210</v>
       </c>
       <c r="J3" t="inlineStr">
@@ -634,7 +637,8 @@
           <t>https://instagram.com/sleepy_dunez</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>{'postUrl': 'https://www.instagram.com/p/DZ5yxYgAy5c/', 'commentUrl': 'https://www.instagram.com/p/DZ5yxYgAy5c/c/17985727140032292', 'id': '17985727140032292', 'text': 'Creo que le deberían cambiar el nombre😭🥀', 'ownerUsername': 'sleepy_dunez', 'ownerProfilePicUrl': 'https://scontent-bru2-1.cdninstagram.com/v/t51.82787-19/726373129_17888033775561289_5001866020940776711_n.jpg?stp=dst-jpg_e0_s150x150_tt6&amp;_nc_cat=110&amp;ig_cache_key=GAmTSytJKuxqEo0-AAeFRSClMmpFbmNDAQAB1501500j-ccb7-5&amp;ccb=7-5&amp;_nc_sid=6</t>
         </is>
@@ -673,7 +677,7 @@
       <c r="H4" s="1" t="n">
         <v>46224.8952199074</v>
       </c>
-      <c r="I4" s="2" t="n">
+      <c r="I4" s="1" t="n">
         <v>46224</v>
       </c>
       <c r="J4" t="inlineStr">
@@ -681,10 +685,8 @@
           <t>21:29:07</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K4" t="n">
+        <v>0</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
@@ -694,7 +696,8 @@
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>{'facebookUrl': 'https://www.facebook.com/100064867445065/posts/pfbid02awSRn7qMHiopGBURJWVj5Yqv6Kxy5dgs7RKPfdZSLYSd2ZUZkJv52cwE582X2XyFl', 'commentUrl': 'https://www.facebook.com/alpina/posts/pfbid02udMVuBcdbK41WvjByhYEQaUDdeSnJEYra5pbSmbpFE35xNrfEPjqpcp5fYfvapznl?comment_id=1726957944992593', 'commentId': '1726957944992593', 'id': 'Y29tbWVudDoxNDc4NTg4MzQ0MzEzNDAwXzE3MjY5NTc5NDQ5OTI1OTM=', 'feedbackId': 'ZmVlZGJhY2s6MTQ3ODU4ODM0NDMxMzQwMF8xNzI2OTU3OTQ0OTkyNTkz', 'date': '2026-07-21T21:29:07.000</t>
         </is>
@@ -733,7 +736,7 @@
       <c r="H5" s="1" t="n">
         <v>46220.97578703704</v>
       </c>
-      <c r="I5" s="2" t="n">
+      <c r="I5" s="1" t="n">
         <v>46220</v>
       </c>
       <c r="J5" t="inlineStr">
@@ -741,10 +744,8 @@
           <t>23:25:08</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="K5" t="n">
+        <v>1</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -754,7 +755,8 @@
       </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr">
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>{'facebookUrl': 'https://www.facebook.com/100064867445065/posts/pfbid02awSRn7qMHiopGBURJWVj5Yqv6Kxy5dgs7RKPfdZSLYSd2ZUZkJv52cwE582X2XyFl', 'commentUrl': 'https://www.facebook.com/alpina/posts/pfbid02udMVuBcdbK41WvjByhYEQaUDdeSnJEYra5pbSmbpFE35xNrfEPjqpcp5fYfvapznl?comment_id=1078533431788344', 'commentId': '1078533431788344', 'id': 'Y29tbWVudDoxNDc4NTg4MzQ0MzEzNDAwXzEwNzg1MzM0MzE3ODgzNDQ=', 'feedbackId': 'ZmVlZGJhY2s6MTQ3ODU4ODM0NDMxMzQwMF8xMDc4NTMzNDMxNzg4MzQ0', 'date': '2026-07-17T23:25:08.000</t>
         </is>
@@ -793,7 +795,7 @@
       <c r="H6" s="1" t="n">
         <v>46224.97891203704</v>
       </c>
-      <c r="I6" s="2" t="n">
+      <c r="I6" s="1" t="n">
         <v>46224</v>
       </c>
       <c r="J6" t="inlineStr">
@@ -801,10 +803,8 @@
           <t>23:29:38</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K6" t="n">
+        <v>0</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
@@ -814,7 +814,8 @@
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr">
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
         <is>
           <t>{'facebookUrl': 'https://www.facebook.com/100064867445065/posts/pfbid0diXSKWcBuTriKjD7Nwt6JVvYPUCCtYhUPBXacCtRb66LmEM7VnPzk5mNx4SPFu81l', 'commentUrl': 'https://www.facebook.com/alpina/posts/pfbid0318dHUiAt3TwtwBAG5K5RTrhvnhqyxZ8twzrn5cnNuYKUiFWwMrvQuCQSuZRsMYpl?comment_id=1037649185543740', 'commentId': '1037649185543740', 'id': 'Y29tbWVudDoxNDgxNTA1MDUwNjg4Mzk2XzEwMzc2NDkxODU1NDM3NDA=', 'feedbackId': 'ZmVlZGJhY2s6MTQ4MTUwNTA1MDY4ODM5Nl8xMDM3NjQ5MTg1NTQzNzQw', 'date': '2026-07-21T23:29:38.000Z'</t>
         </is>
@@ -853,7 +854,7 @@
       <c r="H7" s="1" t="n">
         <v>46223.08563657408</v>
       </c>
-      <c r="I7" s="2" t="n">
+      <c r="I7" s="1" t="n">
         <v>46223</v>
       </c>
       <c r="J7" t="inlineStr">
@@ -861,10 +862,8 @@
           <t>02:03:19</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K7" t="n">
+        <v>0</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -874,7 +873,8 @@
       </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr">
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>{'facebookUrl': 'https://www.facebook.com/100064867445065/posts/pfbid0diXSKWcBuTriKjD7Nwt6JVvYPUCCtYhUPBXacCtRb66LmEM7VnPzk5mNx4SPFu81l', 'commentUrl': 'https://www.facebook.com/alpina/posts/pfbid0318dHUiAt3TwtwBAG5K5RTrhvnhqyxZ8twzrn5cnNuYKUiFWwMrvQuCQSuZRsMYpl?comment_id=1715884343017970', 'commentId': '1715884343017970', 'id': 'Y29tbWVudDoxNDgxNTA1MDUwNjg4Mzk2XzE3MTU4ODQzNDMwMTc5NzA=', 'feedbackId': 'ZmVlZGJhY2s6MTQ4MTUwNTA1MDY4ODM5Nl8xNzE1ODg0MzQzMDE3OTcw', 'date': '2026-07-20T02:03:19.000Z'</t>
         </is>
@@ -913,7 +913,7 @@
       <c r="H8" s="1" t="n">
         <v>46217.89942129629</v>
       </c>
-      <c r="I8" s="2" t="n">
+      <c r="I8" s="1" t="n">
         <v>46217</v>
       </c>
       <c r="J8" t="inlineStr">
@@ -921,10 +921,8 @@
           <t>21:35:10</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K8" t="n">
+        <v>0</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -934,7 +932,8 @@
       </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr">
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>{'facebookUrl': 'https://www.facebook.com/100064867445065/posts/pfbid0diXSKWcBuTriKjD7Nwt6JVvYPUCCtYhUPBXacCtRb66LmEM7VnPzk5mNx4SPFu81l', 'commentUrl': 'https://www.facebook.com/alpina/posts/pfbid0318dHUiAt3TwtwBAG5K5RTrhvnhqyxZ8twzrn5cnNuYKUiFWwMrvQuCQSuZRsMYpl?comment_id=1296257932579939', 'commentId': '1296257932579939', 'id': 'Y29tbWVudDoxNDgxNTA1MDUwNjg4Mzk2XzEyOTYyNTc5MzI1Nzk5Mzk=', 'feedbackId': 'ZmVlZGJhY2s6MTQ4MTUwNTA1MDY4ODM5Nl8xMjk2MjU3OTMyNTc5OTM5', 'date': '2026-07-14T21:35:10.000Z'</t>
         </is>
@@ -973,7 +972,7 @@
       <c r="H9" s="1" t="n">
         <v>46221.04325231481</v>
       </c>
-      <c r="I9" s="2" t="n">
+      <c r="I9" s="1" t="n">
         <v>46221</v>
       </c>
       <c r="J9" t="inlineStr">
@@ -981,10 +980,8 @@
           <t>01:02:17</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K9" t="n">
+        <v>0</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
@@ -994,7 +991,8 @@
       </c>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr">
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>{'facebookUrl': 'https://www.facebook.com/100064867445065/posts/pfbid02jvvAfrhCFmzTnxK1pvNmh15Y8qThsqiWPocQ9dUo3kETV4HhCXc3ZffrAaq4gEHrl', 'commentUrl': 'https://www.facebook.com/alpina/posts/pfbid0PPzCSaFA3zFkaWC8poSXA2EYQuRYnwkjoyLTprPy1r9m2BeiDzFs4vhuxfYak5SUl?comment_id=2000809543966891', 'commentId': '2000809543966891', 'id': 'Y29tbWVudDoxNDc4NjE3NTI0MzEwNDgyXzIwMDA4MDk1NDM5NjY4OTE=', 'feedbackId': 'ZmVlZGJhY2s6MTQ3ODYxNzUyNDMxMDQ4Ml8yMDAwODA5NTQzOTY2ODkx', 'date': '2026-07-18T01:02:17.000Z</t>
         </is>
@@ -1033,7 +1031,7 @@
       <c r="H10" s="1" t="n">
         <v>46221.10013888889</v>
       </c>
-      <c r="I10" s="2" t="n">
+      <c r="I10" s="1" t="n">
         <v>46221</v>
       </c>
       <c r="J10" t="inlineStr">
@@ -1041,10 +1039,8 @@
           <t>02:24:12</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K10" t="n">
+        <v>0</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
@@ -1054,7 +1050,8 @@
       </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr">
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>{'facebookUrl': 'https://www.facebook.com/100064867445065/posts/pfbid02c5QGzXhE2N8V1K1dYhrycRLWmoqMyPgLhkoUWws3WrATKMY3QeVVcgeSE9mTM73Ll', 'commentUrl': 'https://www.facebook.com/alpina/posts/pfbid02nLVXgTHGwmggpBe5faHYc89sSnUpgEdjRFbk5NGY5KGH4PAWPpuk1w7uxjkEhy3ul?comment_id=1570496154770550', 'commentId': '1570496154770550', 'id': 'Y29tbWVudDoxNDgxNTMzMDM3MzUyMjY0XzE1NzA0OTYxNTQ3NzA1NTA=', 'feedbackId': 'ZmVlZGJhY2s6MTQ4MTUzMzAzNzM1MjI2NF8xNTcwNDk2MTU0NzcwNTUw', 'date': '2026-07-18T02:24:12.000</t>
         </is>
@@ -1093,7 +1090,7 @@
       <c r="H11" s="1" t="n">
         <v>46221.00662037037</v>
       </c>
-      <c r="I11" s="2" t="n">
+      <c r="I11" s="1" t="n">
         <v>46221</v>
       </c>
       <c r="J11" t="inlineStr">
@@ -1101,10 +1098,8 @@
           <t>00:09:32</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K11" t="n">
+        <v>0</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
@@ -1114,7 +1109,8 @@
       </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr">
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>{'facebookUrl': 'https://www.facebook.com/100064867445065/posts/pfbid02c5QGzXhE2N8V1K1dYhrycRLWmoqMyPgLhkoUWws3WrATKMY3QeVVcgeSE9mTM73Ll', 'commentUrl': 'https://www.facebook.com/alpina/posts/pfbid02nLVXgTHGwmggpBe5faHYc89sSnUpgEdjRFbk5NGY5KGH4PAWPpuk1w7uxjkEhy3ul?comment_id=2061225511435404', 'commentId': '2061225511435404', 'id': 'Y29tbWVudDoxNDgxNTMzMDM3MzUyMjY0XzIwNjEyMjU1MTE0MzU0MDQ=', 'feedbackId': 'ZmVlZGJhY2s6MTQ4MTUzMzAzNzM1MjI2NF8yMDYxMjI1NTExNDM1NDA0', 'date': '2026-07-18T00:09:32.000</t>
         </is>
@@ -1153,7 +1149,7 @@
       <c r="H12" s="1" t="n">
         <v>46219.06762731481</v>
       </c>
-      <c r="I12" s="2" t="n">
+      <c r="I12" s="1" t="n">
         <v>46219</v>
       </c>
       <c r="J12" t="inlineStr">
@@ -1161,10 +1157,8 @@
           <t>01:37:23</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="K12" t="n">
+        <v>0</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -1174,7 +1168,8 @@
       </c>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr">
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr">
         <is>
           <t>{'facebookUrl': 'https://www.facebook.com/100064867445065/posts/pfbid02c5QGzXhE2N8V1K1dYhrycRLWmoqMyPgLhkoUWws3WrATKMY3QeVVcgeSE9mTM73Ll', 'commentUrl': 'https://www.facebook.com/alpina/posts/pfbid02nLVXgTHGwmggpBe5faHYc89sSnUpgEdjRFbk5NGY5KGH4PAWPpuk1w7uxjkEhy3ul?comment_id=1554955609342819', 'commentId': '1554955609342819', 'id': 'Y29tbWVudDoxNDgxNTMzMDM3MzUyMjY0XzE1NTQ5NTU2MDkzNDI4MTk=', 'feedbackId': 'ZmVlZGJhY2s6MTQ4MTUzMzAzNzM1MjI2NF8xNTU0OTU1NjA5MzQyODE5', 'date': '2026-07-16T01:37:23.000</t>
         </is>

</xml_diff>